<commit_message>
Update Date on Excel file
</commit_message>
<xml_diff>
--- a/Assets/Data/Amstrad/CPC 664/MC0005A/Data CPC 664 MC0005A v2.0.0.xlsx
+++ b/Assets/Data/Amstrad/CPC 664/MC0005A/Data CPC 664 MC0005A v2.0.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbewe\AppData\Local\Classic-Repair-Toolbox\Data\Amstrad\CPC 664\MC0005A\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{986B57A4-96FF-409C-83BC-5D4F6006A4C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6AD8ED4-65CE-4826-B616-4567BB36F17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{EBC5E150-CC27-441B-9E4F-9F7CF77570D6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EBC5E150-CC27-441B-9E4F-9F7CF77570D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Board schematics" sheetId="5" r:id="rId1"/>
@@ -2195,6 +2195,286 @@
     <t>74HCU (High-Speed CMOS Unbuffered): Omits the output buffers, often leaving a single-stage, unbuffered CMOS gate. This results in a more linear input/output characteristic, making it ideal for analogue-like applications such as crystal oscillators and linear amplification</t>
   </si>
   <si>
+    <t>The 8255 operates the keyboard, the sound chip, the cassette recorder but also read links on the PCB. One bit is also used to detect a signal on the expansion port.
+Pin names are associated with the 8255 port i.e. PB0 is Port B bit 0.
+Pin connection is shown in [ ] i.e. Pin 25 PB7 [TAPE RD] is Port B bit 7 connected to the Tape RD signal.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>PB5</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_23_PB5.jpg</t>
+  </si>
+  <si>
+    <t>c64c1bc3-f7c7-4793-a4aa-2412597b109a</t>
+  </si>
+  <si>
+    <t>Input from Expansion Port /EXP pin
+Trace taken with no Expansion connected.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>PB6</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_24_PB6.jpg</t>
+  </si>
+  <si>
+    <t>Input from Parallel/Printer port ready signal.
+Trace taken with no Printer connected.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>PB7</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_25_PB7.jpg</t>
+  </si>
+  <si>
+    <t>08f7b650-c3e4-493b-85b2-b8cdeab6095e</t>
+  </si>
+  <si>
+    <t>d23d6952-243c-490f-b618-0fa2f4067e6b</t>
+  </si>
+  <si>
+    <t>/CS</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_6_CS.jpg</t>
+  </si>
+  <si>
+    <t>3d246aea-f79c-4172-8dea-d2b0776e2d0e</t>
+  </si>
+  <si>
+    <t>Input from A11, low for CS.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Cassette data input
+Trace taken with no Cassette connected.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Input from A9. 
+Confusingly A0 and A1, on the 8255, are not the same as A0 and A1 on the address bus from the Z80 and are connected to A8 and A9 respectively to control which Port is selected on the 8255.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>97508029-f4ae-4370-936b-afd77c36e79c</t>
+  </si>
+  <si>
+    <t>Input from A8. 
+Confusingly A0 and A1, on the 8255, are not the same as A0 and A1 on the address bus from the Z80 and are connected to A8 and A9 respectively to control which Port is selected on the 8255.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>9c622c63-f40d-4360-a52e-21ff023f03f8</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_8_A1.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_9_A0.jpg</t>
+  </si>
+  <si>
+    <t>Input from /IORD.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>4faf6696-9b60-4294-959e-d4948215d028</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_5_RD.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_36_WR.jpg</t>
+  </si>
+  <si>
+    <t>Input from /IOWR.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>RESET</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_35_RESET.jpg</t>
+  </si>
+  <si>
+    <t>Input from RESET.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>e5139825-b588-4a1f-b5f6-bbd7f8f1a996</t>
+  </si>
+  <si>
+    <t>5376bdaf-58fd-4523-817a-7c11293ad1eb</t>
+  </si>
+  <si>
+    <t>PC7</t>
+  </si>
+  <si>
+    <t>6fdac510-bf2b-42af-b165-adb7e4efd176</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_10_PC7.jpg</t>
+  </si>
+  <si>
+    <t>Output to AY BDIR (Bus Direction).
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>PC6</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_11_PC6.jpg</t>
+  </si>
+  <si>
+    <t>Output to AY BC1 (Bus Control).
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>26ff41b1-a6d2-43a1-811d-de37db06229c</t>
+  </si>
+  <si>
+    <t>2a409571-782a-4e7a-96b8-1db2d6dd2210</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_12_PC5.jpg</t>
+  </si>
+  <si>
+    <t>c5e22a9c-7d94-4566-bd6f-5b9a9a6ba116</t>
+  </si>
+  <si>
+    <t>PC5</t>
+  </si>
+  <si>
+    <t>PC4</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_13_PC4.jpg</t>
+  </si>
+  <si>
+    <t>Output to TAPE WR.
+Trace taken with no Cassette connected.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Output to TAPE MOTOR.
+Trace taken with no Cassette connected.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>PA3</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_1_PA3.jpg</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D3.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>43444499-e238-4a7a-af24-5748bd97fc99</t>
+  </si>
+  <si>
+    <t>PA2</t>
+  </si>
+  <si>
+    <t>PA1</t>
+  </si>
+  <si>
+    <t>PA0</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_2_PA2.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_3_PA1.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_4_PA0.jpg</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D2.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D1.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D0.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>9fdb16a6-cbe3-44ff-aa7b-aa444b89c2ac</t>
+  </si>
+  <si>
+    <t>90a516ed-1ecb-48fa-94ee-67553b14520b</t>
+  </si>
+  <si>
+    <t>dd0b875b-4102-4565-802f-e5aaecaaa3c1</t>
+  </si>
+  <si>
+    <t>PA7</t>
+  </si>
+  <si>
+    <t>PA6</t>
+  </si>
+  <si>
+    <t>PA5</t>
+  </si>
+  <si>
+    <t>PA4</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_37_PA7.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_38_PA6.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_39_PA5.jpg</t>
+  </si>
+  <si>
+    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_40_PA4.jpg</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D7.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D6.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D5.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>Input  and Output to AY D4.
+See CPC Wiki for more information.</t>
+  </si>
+  <si>
+    <t>1979c575-4462-4f28-b2df-c1f4adb8fbc5</t>
+  </si>
+  <si>
+    <t>d942f222-5e29-4817-8470-1f6462db78f2</t>
+  </si>
+  <si>
+    <t>c39cf3ec-a302-4830-947d-030ef0efed14</t>
+  </si>
+  <si>
+    <t>58dd292c-a30b-4577-a434-2e1f729dd3c3</t>
+  </si>
+  <si>
+    <t>98e5ea24-504a-47c9-b60a-69e16e88cae0</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve"># Revision date: </t>
     </r>
@@ -2207,288 +2487,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>2026-May-13</t>
+      <t>2026-May-14</t>
     </r>
-  </si>
-  <si>
-    <t>The 8255 operates the keyboard, the sound chip, the cassette recorder but also read links on the PCB. One bit is also used to detect a signal on the expansion port.
-Pin names are associated with the 8255 port i.e. PB0 is Port B bit 0.
-Pin connection is shown in [ ] i.e. Pin 25 PB7 [TAPE RD] is Port B bit 7 connected to the Tape RD signal.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>PB5</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_23_PB5.jpg</t>
-  </si>
-  <si>
-    <t>c64c1bc3-f7c7-4793-a4aa-2412597b109a</t>
-  </si>
-  <si>
-    <t>Input from Expansion Port /EXP pin
-Trace taken with no Expansion connected.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>PB6</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_24_PB6.jpg</t>
-  </si>
-  <si>
-    <t>Input from Parallel/Printer port ready signal.
-Trace taken with no Printer connected.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>PB7</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_25_PB7.jpg</t>
-  </si>
-  <si>
-    <t>08f7b650-c3e4-493b-85b2-b8cdeab6095e</t>
-  </si>
-  <si>
-    <t>d23d6952-243c-490f-b618-0fa2f4067e6b</t>
-  </si>
-  <si>
-    <t>/CS</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_6_CS.jpg</t>
-  </si>
-  <si>
-    <t>3d246aea-f79c-4172-8dea-d2b0776e2d0e</t>
-  </si>
-  <si>
-    <t>Input from A11, low for CS.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Cassette data input
-Trace taken with no Cassette connected.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Input from A9. 
-Confusingly A0 and A1, on the 8255, are not the same as A0 and A1 on the address bus from the Z80 and are connected to A8 and A9 respectively to control which Port is selected on the 8255.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>97508029-f4ae-4370-936b-afd77c36e79c</t>
-  </si>
-  <si>
-    <t>Input from A8. 
-Confusingly A0 and A1, on the 8255, are not the same as A0 and A1 on the address bus from the Z80 and are connected to A8 and A9 respectively to control which Port is selected on the 8255.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>9c622c63-f40d-4360-a52e-21ff023f03f8</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_8_A1.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_9_A0.jpg</t>
-  </si>
-  <si>
-    <t>Input from /IORD.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>4faf6696-9b60-4294-959e-d4948215d028</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_5_RD.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_36_WR.jpg</t>
-  </si>
-  <si>
-    <t>Input from /IOWR.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>RESET</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_35_RESET.jpg</t>
-  </si>
-  <si>
-    <t>Input from RESET.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>e5139825-b588-4a1f-b5f6-bbd7f8f1a996</t>
-  </si>
-  <si>
-    <t>5376bdaf-58fd-4523-817a-7c11293ad1eb</t>
-  </si>
-  <si>
-    <t>PC7</t>
-  </si>
-  <si>
-    <t>6fdac510-bf2b-42af-b165-adb7e4efd176</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_10_PC7.jpg</t>
-  </si>
-  <si>
-    <t>Output to AY BDIR (Bus Direction).
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>PC6</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_11_PC6.jpg</t>
-  </si>
-  <si>
-    <t>Output to AY BC1 (Bus Control).
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>26ff41b1-a6d2-43a1-811d-de37db06229c</t>
-  </si>
-  <si>
-    <t>2a409571-782a-4e7a-96b8-1db2d6dd2210</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_12_PC5.jpg</t>
-  </si>
-  <si>
-    <t>c5e22a9c-7d94-4566-bd6f-5b9a9a6ba116</t>
-  </si>
-  <si>
-    <t>PC5</t>
-  </si>
-  <si>
-    <t>PC4</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_13_PC4.jpg</t>
-  </si>
-  <si>
-    <t>Output to TAPE WR.
-Trace taken with no Cassette connected.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Output to TAPE MOTOR.
-Trace taken with no Cassette connected.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>PA3</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_1_PA3.jpg</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D3.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>43444499-e238-4a7a-af24-5748bd97fc99</t>
-  </si>
-  <si>
-    <t>PA2</t>
-  </si>
-  <si>
-    <t>PA1</t>
-  </si>
-  <si>
-    <t>PA0</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_2_PA2.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_3_PA1.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_4_PA0.jpg</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D2.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D1.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D0.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>9fdb16a6-cbe3-44ff-aa7b-aa444b89c2ac</t>
-  </si>
-  <si>
-    <t>90a516ed-1ecb-48fa-94ee-67553b14520b</t>
-  </si>
-  <si>
-    <t>dd0b875b-4102-4565-802f-e5aaecaaa3c1</t>
-  </si>
-  <si>
-    <t>PA7</t>
-  </si>
-  <si>
-    <t>PA6</t>
-  </si>
-  <si>
-    <t>PA5</t>
-  </si>
-  <si>
-    <t>PA4</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_37_PA7.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_38_PA6.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_39_PA5.jpg</t>
-  </si>
-  <si>
-    <t>Amstrad/CPC 664/MC0005A/Scope baseline/IC107_40_PA4.jpg</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D7.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D6.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D5.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>Input  and Output to AY D4.
-See CPC Wiki for more information.</t>
-  </si>
-  <si>
-    <t>1979c575-4462-4f28-b2df-c1f4adb8fbc5</t>
-  </si>
-  <si>
-    <t>d942f222-5e29-4817-8470-1f6462db78f2</t>
-  </si>
-  <si>
-    <t>c39cf3ec-a302-4830-947d-030ef0efed14</t>
-  </si>
-  <si>
-    <t>58dd292c-a30b-4577-a434-2e1f729dd3c3</t>
-  </si>
-  <si>
-    <t>98e5ea24-504a-47c9-b60a-69e16e88cae0</t>
   </si>
 </sst>
 </file>
@@ -3149,7 +3149,7 @@
     </row>
     <row r="3" spans="1:9" s="8" customFormat="1" ht="21">
       <c r="A3" s="8" t="s">
-        <v>680</v>
+        <v>763</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -5203,7 +5203,7 @@
         <v>542</v>
       </c>
       <c r="J19" s="40" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>350</v>
@@ -5218,7 +5218,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>179</v>
@@ -5233,13 +5233,13 @@
         <v>204</v>
       </c>
       <c r="I20" s="1" t="s">
+        <v>731</v>
+      </c>
+      <c r="J20" s="40" t="s">
         <v>732</v>
       </c>
-      <c r="J20" s="40" t="s">
+      <c r="K20" s="1" t="s">
         <v>733</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>734</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="45">
@@ -5251,7 +5251,7 @@
         <v>2</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>179</v>
@@ -5266,13 +5266,13 @@
         <v>204</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="45">
@@ -5284,7 +5284,7 @@
         <v>3</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>179</v>
@@ -5299,13 +5299,13 @@
         <v>204</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="J22" s="40" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="45">
@@ -5317,7 +5317,7 @@
         <v>4</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>179</v>
@@ -5332,13 +5332,13 @@
         <v>204</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="J23" s="40" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="45">
@@ -5365,13 +5365,13 @@
         <v>204</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="J24" s="40" t="s">
+        <v>704</v>
+      </c>
+      <c r="K24" s="1" t="s">
         <v>705</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="45">
@@ -5383,7 +5383,7 @@
         <v>6</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>179</v>
@@ -5398,13 +5398,13 @@
         <v>204</v>
       </c>
       <c r="I25" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="J25" s="40" t="s">
+        <v>696</v>
+      </c>
+      <c r="K25" s="1" t="s">
         <v>695</v>
-      </c>
-      <c r="J25" s="40" t="s">
-        <v>697</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="105">
@@ -5431,13 +5431,13 @@
         <v>204</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="J26" s="40" t="s">
+        <v>698</v>
+      </c>
+      <c r="K26" s="1" t="s">
         <v>699</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>700</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="105">
@@ -5464,13 +5464,13 @@
         <v>204</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="J27" s="40" t="s">
+        <v>700</v>
+      </c>
+      <c r="K27" s="1" t="s">
         <v>701</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>702</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="45">
@@ -5482,7 +5482,7 @@
         <v>10</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>179</v>
@@ -5497,13 +5497,13 @@
         <v>204</v>
       </c>
       <c r="I28" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="J28" s="40" t="s">
         <v>717</v>
       </c>
-      <c r="J28" s="40" t="s">
-        <v>718</v>
-      </c>
       <c r="K28" s="1" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="45">
@@ -5515,7 +5515,7 @@
         <v>11</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>179</v>
@@ -5530,13 +5530,13 @@
         <v>204</v>
       </c>
       <c r="I29" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="J29" s="40" t="s">
         <v>720</v>
       </c>
-      <c r="J29" s="40" t="s">
+      <c r="K29" s="1" t="s">
         <v>721</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>722</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="75">
@@ -5548,10 +5548,10 @@
         <v>12</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>230</v>
@@ -5563,13 +5563,13 @@
         <v>204</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="J30" s="40" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="75">
@@ -5581,10 +5581,10 @@
         <v>13</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>230</v>
@@ -5596,13 +5596,13 @@
         <v>204</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="J31" s="40" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="30">
@@ -5635,7 +5635,7 @@
         <v>522</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="30">
@@ -5911,10 +5911,10 @@
         <v>23</v>
       </c>
       <c r="D41" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>682</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>683</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>227</v>
@@ -5926,13 +5926,13 @@
         <v>204</v>
       </c>
       <c r="I41" s="1" t="s">
+        <v>683</v>
+      </c>
+      <c r="J41" s="40" t="s">
+        <v>685</v>
+      </c>
+      <c r="K41" s="54" t="s">
         <v>684</v>
-      </c>
-      <c r="J41" s="40" t="s">
-        <v>686</v>
-      </c>
-      <c r="K41" s="54" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="75">
@@ -5944,7 +5944,7 @@
         <v>24</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>519</v>
@@ -5959,13 +5959,13 @@
         <v>204</v>
       </c>
       <c r="I42" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="J42" s="40" t="s">
         <v>688</v>
       </c>
-      <c r="J42" s="40" t="s">
-        <v>689</v>
-      </c>
       <c r="K42" s="54" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="75">
@@ -5977,10 +5977,10 @@
         <v>25</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>227</v>
@@ -5992,13 +5992,13 @@
         <v>204</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="J43" s="40" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="K43" s="54" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="45">
@@ -6010,10 +6010,10 @@
         <v>35</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>227</v>
@@ -6025,13 +6025,13 @@
         <v>204</v>
       </c>
       <c r="I44" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="J44" s="40" t="s">
         <v>711</v>
       </c>
-      <c r="J44" s="40" t="s">
-        <v>712</v>
-      </c>
       <c r="K44" s="54" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="45">
@@ -6058,13 +6058,13 @@
         <v>204</v>
       </c>
       <c r="I45" s="1" t="s">
+        <v>707</v>
+      </c>
+      <c r="J45" s="40" t="s">
         <v>708</v>
       </c>
-      <c r="J45" s="40" t="s">
-        <v>709</v>
-      </c>
       <c r="K45" s="54" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="45">
@@ -6076,7 +6076,7 @@
         <v>37</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>179</v>
@@ -6091,13 +6091,13 @@
         <v>204</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="J46" s="40" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="45">
@@ -6109,7 +6109,7 @@
         <v>38</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>179</v>
@@ -6124,13 +6124,13 @@
         <v>204</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="J47" s="40" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="45">
@@ -6142,7 +6142,7 @@
         <v>39</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>179</v>
@@ -6157,13 +6157,13 @@
         <v>204</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="J48" s="40" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="45">
@@ -6175,7 +6175,7 @@
         <v>40</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>179</v>
@@ -6190,13 +6190,13 @@
         <v>204</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="J49" s="40" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="45">

</xml_diff>